<commit_message>
streeteasy report: full data points per listing in PDF; deposit fix
Landscape PDF with a 17-column index table and per-listing sections
carrying every captured field (IDs, dates, baths breakdown, lease
terms, broker license/address, fees, price + unit history, media,
coordinates, full description). Security deposit now derived from
the move-in fee schedule when the pricing field is null (27/31
filled); flows through xlsx and map too.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VTc6fULb99AoJrKNCxkHhF
</commit_message>
<xml_diff>
--- a/personal/streeteasy-2026-07-12/streeteasy_listings_2026-07-12.xlsx
+++ b/personal/streeteasy-2026-07-12/streeteasy_listings_2026-07-12.xlsx
@@ -965,7 +965,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN2" s="4" t="n"/>
+      <c r="AN2" s="4" t="n">
+        <v>6995</v>
+      </c>
       <c r="AO2" s="5" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $6,995</t>
@@ -1209,7 +1211,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN3" s="8" t="n"/>
+      <c r="AN3" s="8" t="n">
+        <v>7995</v>
+      </c>
       <c r="AO3" s="9" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $7,995</t>
@@ -1410,7 +1414,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN4" s="4" t="n"/>
+      <c r="AN4" s="4" t="n">
+        <v>7995</v>
+      </c>
       <c r="AO4" s="5" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $7,995</t>
@@ -1616,7 +1622,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN5" s="8" t="n"/>
+      <c r="AN5" s="8" t="n">
+        <v>7995</v>
+      </c>
       <c r="AO5" s="9" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $7,995</t>
@@ -1821,7 +1829,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN6" s="4" t="n"/>
+      <c r="AN6" s="4" t="n">
+        <v>8995</v>
+      </c>
       <c r="AO6" s="5" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $8,995</t>
@@ -2006,7 +2016,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN7" s="8" t="n"/>
+      <c r="AN7" s="8" t="n">
+        <v>9500</v>
+      </c>
       <c r="AO7" s="9" t="inlineStr">
         <is>
           <t>Application fee: $300; Background check: $50; Security deposit: $9,500; Early termination: $9,500</t>
@@ -2229,7 +2241,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN8" s="4" t="n"/>
+      <c r="AN8" s="4" t="n">
+        <v>10600</v>
+      </c>
       <c r="AO8" s="5" t="inlineStr">
         <is>
           <t>Application fee: $20; Pet deposit: $250; Security deposit: $10,600; Bike storage: $15; Community amenity: $50; Storage: $50</t>
@@ -2436,7 +2450,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN9" s="8" t="n"/>
+      <c r="AN9" s="8" t="n">
+        <v>12500</v>
+      </c>
       <c r="AO9" s="9" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $12,500</t>
@@ -2643,7 +2659,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN10" s="4" t="n"/>
+      <c r="AN10" s="4" t="n">
+        <v>13400</v>
+      </c>
       <c r="AO10" s="5" t="inlineStr">
         <is>
           <t>Administration: $17; Application fee: $20; Security deposit: $13,400</t>
@@ -2843,7 +2861,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN11" s="8" t="n"/>
+      <c r="AN11" s="8" t="n">
+        <v>14750</v>
+      </c>
       <c r="AO11" s="9" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $14,750</t>
@@ -3048,7 +3068,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN12" s="4" t="n"/>
+      <c r="AN12" s="4" t="n">
+        <v>8300</v>
+      </c>
       <c r="AO12" s="5" t="inlineStr">
         <is>
           <t>Application fee: $0; Security deposit: $8,300</t>
@@ -3257,7 +3279,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN13" s="8" t="n"/>
+      <c r="AN13" s="8" t="n">
+        <v>10850</v>
+      </c>
       <c r="AO13" s="9" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $10,850</t>
@@ -3490,7 +3514,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN14" s="4" t="n"/>
+      <c r="AN14" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="AO14" s="5" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $0</t>
@@ -3697,7 +3723,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN15" s="8" t="n"/>
+      <c r="AN15" s="8" t="n">
+        <v>18000</v>
+      </c>
       <c r="AO15" s="9" t="inlineStr">
         <is>
           <t>Move-in deposit: $500; Application fee: $0; Security deposit: $18,000</t>
@@ -3901,7 +3929,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN16" s="4" t="n"/>
+      <c r="AN16" s="4" t="n">
+        <v>18000</v>
+      </c>
       <c r="AO16" s="5" t="inlineStr">
         <is>
           <t>Application fee: $18,000; Security deposit: $18,000</t>
@@ -4136,7 +4166,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN17" s="8" t="n"/>
+      <c r="AN17" s="8" t="n">
+        <v>6995</v>
+      </c>
       <c r="AO17" s="9" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $6,995</t>
@@ -4362,7 +4394,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN18" s="4" t="n"/>
+      <c r="AN18" s="4" t="n">
+        <v>8250</v>
+      </c>
       <c r="AO18" s="5" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $8,250</t>
@@ -4752,7 +4786,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN20" s="4" t="n"/>
+      <c r="AN20" s="4" t="n">
+        <v>12000</v>
+      </c>
       <c r="AO20" s="5" t="inlineStr">
         <is>
           <t>Application fee: $0; Security deposit: $12,000; Credit check: $20</t>
@@ -4948,7 +4984,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN21" s="8" t="n"/>
+      <c r="AN21" s="8" t="n">
+        <v>16500</v>
+      </c>
       <c r="AO21" s="9" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $16,500</t>
@@ -5715,7 +5753,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN25" s="8" t="n"/>
+      <c r="AN25" s="8" t="n">
+        <v>8995</v>
+      </c>
       <c r="AO25" s="9" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $8,995</t>
@@ -5926,7 +5966,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN26" s="4" t="n"/>
+      <c r="AN26" s="4" t="n">
+        <v>4750</v>
+      </c>
       <c r="AO26" s="5" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $4,750</t>
@@ -6127,7 +6169,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN27" s="8" t="n"/>
+      <c r="AN27" s="8" t="n">
+        <v>4997.5</v>
+      </c>
       <c r="AO27" s="9" t="inlineStr">
         <is>
           <t>Move-in fee: $80; Application fee: $20; Key replacement: $75; Security deposit: $4,998</t>
@@ -6337,7 +6381,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN28" s="4" t="n"/>
+      <c r="AN28" s="4" t="n">
+        <v>11995</v>
+      </c>
       <c r="AO28" s="5" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $11,995</t>
@@ -6534,7 +6580,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN29" s="8" t="n"/>
+      <c r="AN29" s="8" t="n">
+        <v>5997.5</v>
+      </c>
       <c r="AO29" s="9" t="inlineStr">
         <is>
           <t>Move-in fee: $80; Application fee: $20; Key replacement: $75; Security deposit: $5,998</t>
@@ -6750,7 +6798,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN30" s="4" t="n"/>
+      <c r="AN30" s="4" t="n">
+        <v>12500</v>
+      </c>
       <c r="AO30" s="5" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $12,500</t>
@@ -6955,7 +7005,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN31" s="8" t="n"/>
+      <c r="AN31" s="8" t="n">
+        <v>14000</v>
+      </c>
       <c r="AO31" s="9" t="inlineStr">
         <is>
           <t>Application fee: $0; Security deposit: $14,000</t>
@@ -7164,7 +7216,9 @@
           <t>None listed</t>
         </is>
       </c>
-      <c r="AN32" s="4" t="n"/>
+      <c r="AN32" s="4" t="n">
+        <v>16999</v>
+      </c>
       <c r="AO32" s="5" t="inlineStr">
         <is>
           <t>Application fee: $20; Security deposit: $16,999</t>

</xml_diff>